<commit_message>
generate normal metrics to jitter realistic baseline values
</commit_message>
<xml_diff>
--- a/Project_timeline.xlsx
+++ b/Project_timeline.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\users\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\devops-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46078A62-97FC-4F60-8B25-892C19BE1885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4B670F-2974-4917-A3B0-F7A0CCE57C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,9 +37,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="84">
   <si>
-    <t>🛡️ SENTINEL AI — DevOps Incident Response Agent | Project Timeline</t>
-  </si>
-  <si>
     <t>Project Start: 25-Apr-2026  |  Duration: 10 working days  |  Owner: Data Scientist (Personal Project)</t>
   </si>
   <si>
@@ -287,6 +284,9 @@
   </si>
   <si>
     <t>Phase-Level Summary</t>
+  </si>
+  <si>
+    <t>SENTINEL AI — DevOps Incident Response Agent | Project Timeline</t>
   </si>
 </sst>
 </file>
@@ -466,128 +466,128 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -864,406 +864,412 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
+      <c r="A1" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
     </row>
     <row r="2" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+    </row>
+    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="37" t="s">
-        <v>82</v>
-      </c>
-      <c r="G4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="F5" s="7">
+        <v>1</v>
+      </c>
+      <c r="G5" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="8">
+      <c r="C6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="7">
         <v>0.5</v>
       </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="F6" s="7">
+        <v>2</v>
+      </c>
+      <c r="G6" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="8">
+      <c r="B7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="7">
+        <v>1</v>
+      </c>
+      <c r="F7" s="7">
+        <v>6</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="7">
+        <v>1</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="13">
+        <v>1</v>
+      </c>
+      <c r="F9" s="13"/>
+      <c r="G9" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="13">
+        <v>1</v>
+      </c>
+      <c r="F10" s="13"/>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="13">
+        <v>1</v>
+      </c>
+      <c r="F11" s="13"/>
+      <c r="G11" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="13">
+        <v>1</v>
+      </c>
+      <c r="F12" s="13"/>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="19">
         <v>0.5</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="8">
+      <c r="F13" s="19"/>
+      <c r="G13" s="20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="25">
         <v>1</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" s="8">
+      <c r="F15" s="25"/>
+      <c r="G15" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" s="25">
         <v>1</v>
       </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="14">
+      <c r="F16" s="25"/>
+      <c r="G16" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="25">
         <v>1</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="14">
-        <v>1</v>
-      </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="14">
-        <v>1</v>
-      </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="14">
-        <v>1</v>
-      </c>
-      <c r="F12" s="14"/>
-      <c r="G12" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="F13" s="20"/>
-      <c r="G13" s="21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="E14" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="F14" s="20"/>
-      <c r="G14" s="21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="E15" s="26">
-        <v>1</v>
-      </c>
-      <c r="F15" s="26"/>
-      <c r="G15" s="27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="E16" s="26">
-        <v>1</v>
-      </c>
-      <c r="F16" s="26"/>
-      <c r="G16" s="27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="D17" s="25" t="s">
+      <c r="F17" s="25"/>
+      <c r="G17" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="26">
-        <v>1</v>
-      </c>
-      <c r="F17" s="26"/>
-      <c r="G17" s="27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="28" t="s">
+      <c r="B18" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="C18" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="30" t="s">
+      <c r="D18" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="31" t="s">
+      <c r="E18" s="31">
+        <v>0.3</v>
+      </c>
+      <c r="F18" s="31"/>
+      <c r="G18" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="E18" s="32">
+      <c r="C19" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19" s="31">
+        <v>0.4</v>
+      </c>
+      <c r="F19" s="31"/>
+      <c r="G19" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="E20" s="31">
         <v>0.3</v>
       </c>
-      <c r="F18" s="32"/>
-      <c r="G18" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>62</v>
-      </c>
-      <c r="E19" s="32">
-        <v>0.4</v>
-      </c>
-      <c r="F19" s="32"/>
-      <c r="G19" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" s="31" t="s">
+      <c r="F20" s="31"/>
+      <c r="G20" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="32">
-        <v>0.3</v>
-      </c>
-      <c r="F20" s="32"/>
-      <c r="G20" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="34" t="s">
+      <c r="B21" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="34">
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="1">
         <f>SUM(E5:E20)</f>
         <v>12.000000000000002</v>
       </c>
-      <c r="F21" s="34">
+      <c r="F21" s="1">
         <f>SUM(F5:F20)</f>
-        <v>0</v>
-      </c>
-      <c r="G21" s="35">
+        <v>9</v>
+      </c>
+      <c r="G21" s="33">
         <f>AVERAGE(G5:G20)</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
   </sheetData>
@@ -1288,122 +1294,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
-        <v>83</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
+      <c r="A1" s="40" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
     </row>
     <row r="3" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="E3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="34" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="E3" s="34" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="38" t="s">
+      <c r="B4" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="7">
+        <v>3</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="8">
+      <c r="B5" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="13">
+        <v>4</v>
+      </c>
+      <c r="D5" s="13"/>
+      <c r="E5" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="37" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="19">
+        <v>1</v>
+      </c>
+      <c r="D6" s="19"/>
+      <c r="E6" s="20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="38" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="25">
         <v>3</v>
       </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="39" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="14">
-        <v>4</v>
-      </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="40" t="s">
-        <v>75</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="20">
+      <c r="D7" s="25"/>
+      <c r="E7" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="39" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="31">
         <v>1</v>
       </c>
-      <c r="D6" s="20"/>
-      <c r="E6" s="21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="41" t="s">
-        <v>77</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="26">
-        <v>3</v>
-      </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="42" t="s">
-        <v>79</v>
-      </c>
-      <c r="B8" s="28" t="s">
+      <c r="D8" s="31"/>
+      <c r="E8" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="32">
-        <v>1</v>
-      </c>
-      <c r="D8" s="32"/>
-      <c r="E8" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
-        <v>66</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" s="34">
+      <c r="C9" s="1">
         <f>SUM(C4:C8)</f>
         <v>12</v>
       </c>
-      <c r="D9" s="34">
+      <c r="D9" s="1">
         <f>SUM(D4:D8)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="35">
+      <c r="E9" s="33">
         <f>AVERAGE(E4:E8)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Initialize memory (not completed yet)
</commit_message>
<xml_diff>
--- a/Project_timeline.xlsx
+++ b/Project_timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\devops-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4B670F-2974-4917-A3B0-F7A0CCE57C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE7CA1CE-3444-4E89-99E0-8D39B06739F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Timeline" sheetId="1" r:id="rId1"/>
@@ -100,9 +100,6 @@
     <t>Implement DB connection pool exhaustion, memory leak in auth-service, and cascading failure scenarios in incidents.py with realistic symptom evolution. Add incident_injector to trigger them on demand.</t>
   </si>
   <si>
-    <t>27-Apr-2026 (Mon)</t>
-  </si>
-  <si>
     <t>LangGraph Orchestrator</t>
   </si>
   <si>
@@ -287,6 +284,9 @@
   </si>
   <si>
     <t>SENTINEL AI — DevOps Incident Response Agent | Project Timeline</t>
+  </si>
+  <si>
+    <t>10-May-2026 (Sun)</t>
   </si>
 </sst>
 </file>
@@ -865,7 +865,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -902,7 +902,7 @@
         <v>5</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>6</v>
@@ -974,12 +974,12 @@
         <v>6</v>
       </c>
       <c r="G7" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>18</v>
@@ -993,44 +993,48 @@
       <c r="E8" s="7">
         <v>1</v>
       </c>
-      <c r="F8" s="7"/>
+      <c r="F8" s="7">
+        <v>1</v>
+      </c>
       <c r="G8" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="C9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="12" t="s">
-        <v>24</v>
-      </c>
       <c r="E9" s="13">
         <v>1</v>
       </c>
-      <c r="F9" s="13"/>
+      <c r="F9" s="13">
+        <v>2</v>
+      </c>
       <c r="G9" s="14">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="C10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="D10" s="12" t="s">
         <v>27</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>28</v>
       </c>
       <c r="E10" s="13">
         <v>1</v>
@@ -1042,16 +1046,16 @@
     </row>
     <row r="11" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="C11" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="D11" s="12" t="s">
         <v>31</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>32</v>
       </c>
       <c r="E11" s="13">
         <v>1</v>
@@ -1063,16 +1067,16 @@
     </row>
     <row r="12" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="D12" s="12" t="s">
         <v>34</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>35</v>
       </c>
       <c r="E12" s="13">
         <v>1</v>
@@ -1084,16 +1088,16 @@
     </row>
     <row r="13" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="C13" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="D13" s="18" t="s">
         <v>38</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>39</v>
       </c>
       <c r="E13" s="19">
         <v>0.5</v>
@@ -1105,16 +1109,16 @@
     </row>
     <row r="14" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="D14" s="18" t="s">
         <v>41</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>42</v>
       </c>
       <c r="E14" s="19">
         <v>0.5</v>
@@ -1126,16 +1130,16 @@
     </row>
     <row r="15" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="C15" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="D15" s="24" t="s">
         <v>45</v>
-      </c>
-      <c r="D15" s="24" t="s">
-        <v>46</v>
       </c>
       <c r="E15" s="25">
         <v>1</v>
@@ -1147,16 +1151,16 @@
     </row>
     <row r="16" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="C16" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="D16" s="24" t="s">
         <v>49</v>
-      </c>
-      <c r="D16" s="24" t="s">
-        <v>50</v>
       </c>
       <c r="E16" s="25">
         <v>1</v>
@@ -1168,16 +1172,16 @@
     </row>
     <row r="17" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="C17" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="D17" s="24" t="s">
         <v>53</v>
-      </c>
-      <c r="D17" s="24" t="s">
-        <v>54</v>
       </c>
       <c r="E17" s="25">
         <v>1</v>
@@ -1189,16 +1193,16 @@
     </row>
     <row r="18" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="28" t="s">
+      <c r="C18" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="D18" s="30" t="s">
         <v>57</v>
-      </c>
-      <c r="D18" s="30" t="s">
-        <v>58</v>
       </c>
       <c r="E18" s="31">
         <v>0.3</v>
@@ -1210,16 +1214,16 @@
     </row>
     <row r="19" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B19" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="D19" s="30" t="s">
         <v>60</v>
-      </c>
-      <c r="D19" s="30" t="s">
-        <v>61</v>
       </c>
       <c r="E19" s="31">
         <v>0.4</v>
@@ -1231,16 +1235,16 @@
     </row>
     <row r="20" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B20" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="D20" s="30" t="s">
         <v>63</v>
-      </c>
-      <c r="D20" s="30" t="s">
-        <v>64</v>
       </c>
       <c r="E20" s="31">
         <v>0.3</v>
@@ -1252,10 +1256,10 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="42" t="s">
         <v>65</v>
-      </c>
-      <c r="B21" s="42" t="s">
-        <v>66</v>
       </c>
       <c r="C21" s="42"/>
       <c r="D21" s="42"/>
@@ -1265,11 +1269,11 @@
       </c>
       <c r="F21" s="1">
         <f>SUM(F5:F20)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G21" s="33">
         <f>AVERAGE(G5:G20)</f>
-        <v>0.125</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>
@@ -1295,7 +1299,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="40" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -1304,16 +1308,16 @@
     </row>
     <row r="3" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>68</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>6</v>
@@ -1321,10 +1325,10 @@
     </row>
     <row r="4" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="C4" s="7">
         <v>3</v>
@@ -1336,10 +1340,10 @@
     </row>
     <row r="5" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>73</v>
       </c>
       <c r="C5" s="13">
         <v>4</v>
@@ -1351,10 +1355,10 @@
     </row>
     <row r="6" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>74</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>75</v>
       </c>
       <c r="C6" s="19">
         <v>1</v>
@@ -1366,10 +1370,10 @@
     </row>
     <row r="7" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="21" t="s">
         <v>76</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>77</v>
       </c>
       <c r="C7" s="25">
         <v>3</v>
@@ -1381,10 +1385,10 @@
     </row>
     <row r="8" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="27" t="s">
         <v>78</v>
-      </c>
-      <c r="B8" s="27" t="s">
-        <v>79</v>
       </c>
       <c r="C8" s="31">
         <v>1</v>
@@ -1396,10 +1400,10 @@
     </row>
     <row r="9" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C9" s="1">
         <f>SUM(C4:C8)</f>

</xml_diff>